<commit_message>
DataCleaner->RouteInfoParser+усиление.IDManagerDialog удаление ID_car,MenuBar,StartupSplash,изменения CreateRaceDialog
</commit_message>
<xml_diff>
--- a/LogistX/config/1c_unclosed_races.xlsx
+++ b/LogistX/config/1c_unclosed_races.xlsx
@@ -413,16 +413,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="46" customWidth="1" min="3" max="3"/>
     <col width="38" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -465,7 +465,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>АКБ № 1</t>
+          <t>АКБ № 2</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -483,32 +483,156 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>С 501 МВ 716 SITRAK C7H 4X2 MAX</t>
+          <t>Х 746 ТН 790 SITRAK ZZ4186V391HE</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Рейс (уэ) ВТ000009671 от 29.06.2026 12:17:07</t>
+          <t>Рейс (уэ) ВТ000009827 от 02.07.2026 10:27:46</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>05.07.2026 15:00:00</t>
+          <t>08.07.2026 14:00:00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Новосибирская обл., г. Новосибирск, п. Садовый, ул. Пасечная, д. 1 Б, к. 1</t>
+          <t>Новосибирская обл., г. Обь, ул. 3307-й км, д. 16, к. 8</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Хабаровский край, Хабаровский р-н, с. Ракитное, пр-д Перспективный, д. 3 А</t>
+          <t>Амурская обл., г. Благовещенск, п. Астрахановка, ул. Полевая, д. 50/1</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>Интернет Решения</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>В 295 АС 250 SANY 495AS</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Рейс (уэ) ДВ000001246 от 07.07.2026 9:20:31</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>08.07.2026 14:00:00</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Московская обл., г. Домодедово, мкр. Белые Столбы, вл. Склады 104, с. 4/1</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Вологодская обл., г. Вологда, ш. Окружное, д. 13</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>РВБ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>АКБ № 3</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>М 323 КХ 790 SCANIA (R4X200 R 450)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Рейс (уэ) ВТ000009927 от 03.07.2026 15:11:57</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>08.07.2026 14:00:00</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Московская обл., г. Домодедово, мкр Северный, ул. Логистическая, д. 1/7</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Новосибирская обл., г. Новосибирск, пр-д Энергетиков, д. 17</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>МТП (Мейджик Транс Поволжье - ДК ЛОРД)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>О 263 УУ 790 SITRAK ZZ4186V391HE</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Рейс (уэ) ВЕ000001077 от 26.06.2026 10:51:56</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>08.07.2026 14:00:00</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Приморский край, г. Уссурийск, ул. Коммунальная, д. 5 Б</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Москва, г. Москва, 19 -й км Южные Ворота</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>ТРНСК</t>
         </is>
       </c>
     </row>

</xml_diff>